<commit_message>
Bilan 2025 : les quatre avis d'echeance AG Insurance sont coches
Police 037524039 : 431,25 en janvier et avril, 458,66 en juillet et
octobre, soit 1.779,82. Avancement : 98,1 %.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1026,18 +1026,22 @@
       <c r="F13" s="17" t="n"/>
       <c r="G13" s="31" t="n"/>
       <c r="H13" s="32" t="n"/>
-      <c r="I13" s="33" t="inlineStr">
+      <c r="I13" s="13" t="inlineStr">
         <is>
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J13" s="34" t="n">
+      <c r="J13" s="37" t="n">
         <v>431.25</v>
       </c>
-      <c r="K13" s="35" t="n"/>
-      <c r="L13" s="36" t="inlineStr">
-        <is>
-          <t>Paiement par domiciliation (AG Insurance)</t>
+      <c r="K13" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L13" s="32" t="inlineStr">
+        <is>
+          <t>Paiement par domiciliation (AG Insurance) — Avis d'échéance AG Insurance en main — police 037524039</t>
         </is>
       </c>
     </row>
@@ -3908,18 +3912,22 @@
       <c r="F138" s="17" t="n"/>
       <c r="G138" s="31" t="n"/>
       <c r="H138" s="32" t="n"/>
-      <c r="I138" s="33" t="inlineStr">
+      <c r="I138" s="13" t="inlineStr">
         <is>
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J138" s="34" t="n">
+      <c r="J138" s="37" t="n">
         <v>431.25</v>
       </c>
-      <c r="K138" s="35" t="n"/>
-      <c r="L138" s="36" t="inlineStr">
-        <is>
-          <t>Paiement par domiciliation (AG Insurance)</t>
+      <c r="K138" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L138" s="32" t="inlineStr">
+        <is>
+          <t>Paiement par domiciliation (AG Insurance) — Avis d'échéance AG Insurance en main — police 037524039</t>
         </is>
       </c>
     </row>
@@ -7074,18 +7082,22 @@
       <c r="F277" s="17" t="n"/>
       <c r="G277" s="31" t="n"/>
       <c r="H277" s="32" t="n"/>
-      <c r="I277" s="33" t="inlineStr">
+      <c r="I277" s="13" t="inlineStr">
         <is>
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J277" s="34" t="n">
+      <c r="J277" s="37" t="n">
         <v>458.66</v>
       </c>
-      <c r="K277" s="35" t="n"/>
-      <c r="L277" s="36" t="inlineStr">
-        <is>
-          <t>Domiciliation AG Insurance — prime passée de 431,25 à 458,66</t>
+      <c r="K277" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L277" s="32" t="inlineStr">
+        <is>
+          <t>Domiciliation AG Insurance — prime passée de 431,25 à 458,66 — Avis d'échéance AG Insurance en main — police 037524039</t>
         </is>
       </c>
     </row>
@@ -9652,18 +9664,22 @@
       <c r="F389" s="17" t="n"/>
       <c r="G389" s="31" t="n"/>
       <c r="H389" s="32" t="n"/>
-      <c r="I389" s="33" t="inlineStr">
+      <c r="I389" s="13" t="inlineStr">
         <is>
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J389" s="34" t="n">
+      <c r="J389" s="37" t="n">
         <v>458.66</v>
       </c>
-      <c r="K389" s="35" t="n"/>
-      <c r="L389" s="36" t="inlineStr">
-        <is>
-          <t>Paiement par domiciliation (AG Insurance)</t>
+      <c r="K389" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L389" s="32" t="inlineStr">
+        <is>
+          <t>Paiement par domiciliation (AG Insurance) — Avis d'échéance AG Insurance en main — police 037524039</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : la quittance LRS Insurance est cochee
RC professionnelle, 55,04 payee le 16-12-2025.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -11112,18 +11112,22 @@
       <c r="F452" s="17" t="n"/>
       <c r="G452" s="31" t="n"/>
       <c r="H452" s="32" t="n"/>
-      <c r="I452" s="33" t="inlineStr">
+      <c r="I452" s="13" t="inlineStr">
         <is>
           <t>Assurance RC - LRS Insurance</t>
         </is>
       </c>
-      <c r="J452" s="34" t="n">
+      <c r="J452" s="37" t="n">
         <v>55.04</v>
       </c>
-      <c r="K452" s="35" t="n"/>
-      <c r="L452" s="36" t="inlineStr">
-        <is>
-          <t>RC professionnelle — prime annuelle payée le 16-12-2025, communication 025/0074/58347. Même montant qu'en 2024, où le courtier était Liantis</t>
+      <c r="K452" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L452" s="32" t="inlineStr">
+        <is>
+          <t>RC professionnelle — prime annuelle payée le 16-12-2025, communication 025/0074/58347. Même montant qu'en 2024, où le courtier était Liantis — Quittance LRS Insurance en main — RC professionnelle</t>
         </is>
       </c>
     </row>

</xml_diff>